<commit_message>
chore: weekly briefing 2026-10-02 23:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-09-28.xlsx
+++ b/public/reports/weekly_briefing/2026-09-28.xlsx
@@ -1031,7 +1031,7 @@
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>미국 종가 기준 09/25 → 10/01, %</t>
+          <t>미국 종가 기준 09/25 → 10/02, %</t>
         </is>
       </c>
       <c r="I6" s="18" t="inlineStr"/>
@@ -1101,19 +1101,19 @@
         <v>-9531</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>-0.99</v>
+        <v>-0.27</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>-1.74</v>
-      </c>
-      <c r="G8" s="29" t="n">
-        <v>-0.73</v>
+        <v>-1.26</v>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>0.45</v>
       </c>
       <c r="H8" s="28" t="n">
-        <v>10.22</v>
+        <v>2.96</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>1.26</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="9">
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="D12" s="32" t="n">
-        <v>1.85</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="13">
@@ -1188,11 +1188,11 @@
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
-          <t>에너지</t>
+          <t>기술</t>
         </is>
       </c>
       <c r="D13" s="32" t="n">
-        <v>1.06</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="14">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C14" s="31" t="inlineStr">
         <is>
-          <t>기술</t>
+          <t>에너지</t>
         </is>
       </c>
       <c r="D14" s="32" t="n">
-        <v>0.78</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="15">
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="D15" s="33" t="n">
-        <v>-2.64</v>
+        <v>-2.65</v>
       </c>
     </row>
     <row r="16">
@@ -1248,11 +1248,11 @@
       </c>
       <c r="C16" s="31" t="inlineStr">
         <is>
-          <t>소재</t>
+          <t>금융</t>
         </is>
       </c>
       <c r="D16" s="33" t="n">
-        <v>-2.53</v>
+        <v>-2.46</v>
       </c>
     </row>
     <row r="17">
@@ -1268,11 +1268,11 @@
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>금융</t>
+          <t>소재</t>
         </is>
       </c>
       <c r="D17" s="33" t="n">
-        <v>-2.52</v>
+        <v>-1.89</v>
       </c>
     </row>
     <row r="18">
@@ -12229,7 +12229,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8580FB53-DE1B-4360-9D73-FBA788AC55D3}</x14:id>
+          <x14:id>{3F2172BB-0113-4C09-AE1F-623CCABF29F5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12243,7 +12243,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2929D69C-5216-416A-B0B2-733D94529FFB}</x14:id>
+          <x14:id>{8DAFD477-6F51-4779-9D43-3E70D36F0A7C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12257,7 +12257,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E7DDFEC0-5C82-4BA5-BA55-57A1326F11BD}</x14:id>
+          <x14:id>{718A2435-64E9-424D-B4B6-DF3C05ED8EB6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12271,7 +12271,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{095E8FB3-7D77-4E69-BB4C-F771AB97A1A4}</x14:id>
+          <x14:id>{4C06611F-2AE3-4C61-9D3D-641F18229063}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12281,7 +12281,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8580FB53-DE1B-4360-9D73-FBA788AC55D3}">
+          <x14:cfRule type="dataBar" id="{3F2172BB-0113-4C09-AE1F-623CCABF29F5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12294,7 +12294,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2929D69C-5216-416A-B0B2-733D94529FFB}">
+          <x14:cfRule type="dataBar" id="{8DAFD477-6F51-4779-9D43-3E70D36F0A7C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12307,7 +12307,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E7DDFEC0-5C82-4BA5-BA55-57A1326F11BD}">
+          <x14:cfRule type="dataBar" id="{718A2435-64E9-424D-B4B6-DF3C05ED8EB6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12320,7 +12320,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{095E8FB3-7D77-4E69-BB4C-F771AB97A1A4}">
+          <x14:cfRule type="dataBar" id="{4C06611F-2AE3-4C61-9D3D-641F18229063}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>